<commit_message>
feat: add Kayla Zuhrotun Nisa achievement record in English competition at National level (Juara 2)
</commit_message>
<xml_diff>
--- a/lomba/lomba.xlsx
+++ b/lomba/lomba.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\hibatullah iibs\lomba\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\website hibatullah\lomba\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B28853CE-B1FA-4128-BA65-9FFFAE8665D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA159E33-1D0C-41D0-8C72-B063EB8B89AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11295" xr2:uid="{026E4CFC-AFE7-407D-8063-5B2F99C64B8C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{026E4CFC-AFE7-407D-8063-5B2F99C64B8C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,21 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="14">
   <si>
     <t>Nama Santri</t>
   </si>
@@ -67,6 +58,15 @@
   </si>
   <si>
     <t>Kabupaten</t>
+  </si>
+  <si>
+    <t>kayla  zuhrotun nisa</t>
+  </si>
+  <si>
+    <t>Nasional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bahasa inggris </t>
   </si>
 </sst>
 </file>
@@ -162,7 +162,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -171,14 +171,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -523,7 +522,7 @@
       <c r="B2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D2" s="3">
@@ -537,7 +536,7 @@
       <c r="B3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D3" s="3">
@@ -551,7 +550,7 @@
       <c r="B4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D4" s="3">
@@ -559,13 +558,13 @@
       </c>
     </row>
     <row r="5" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="3">
@@ -573,21 +572,32 @@
       </c>
     </row>
     <row r="6" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="3">
         <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C7" s="6"/>
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="3">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>